<commit_message>
Fix report export alignment and Location column overflow
Claiming kW/h and Rate kW/h were right-aligned (default for numeric
cells) while their header-block peers are left-aligned text; the
Location column was too narrow for real addresses, so long values
spilled past the table's border into blank cells instead of wrapping.
</commit_message>
<xml_diff>
--- a/static/templates/home-charging-template.xlsx
+++ b/static/templates/home-charging-template.xlsx
@@ -175,22 +175,37 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -543,7 +558,7 @@
     <col min="2" max="2" width="16" customWidth="1"/>
     <col min="3" max="3" width="14" customWidth="1"/>
     <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="26" customWidth="1"/>
+    <col min="5" max="5" width="40" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -616,7 +631,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>14</v>
       </c>
@@ -629,11 +644,11 @@
       <c r="D8" s="10">
         <v>8.2</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="11" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
         <v>16</v>
       </c>
@@ -646,11 +661,11 @@
       <c r="D9" s="10">
         <v>7.9</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="11" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
         <v>17</v>
       </c>
@@ -663,27 +678,27 @@
       <c r="D10" s="10">
         <v>9.1</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="11" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="11" t="s">
+      <c r="A11" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="11"/>
-      <c r="C11" s="11"/>
-      <c r="D11" s="12">
+      <c r="B11" s="12"/>
+      <c r="C11" s="12"/>
+      <c r="D11" s="13">
         <f>SUM(D8:D10)</f>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="11" t="s">
+      <c r="A12" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B12" s="11"/>
-      <c r="C12" s="11"/>
-      <c r="D12" s="13">
+      <c r="B12" s="12"/>
+      <c r="C12" s="12"/>
+      <c r="D12" s="14">
         <f>D11*E4</f>
       </c>
     </row>
@@ -713,7 +728,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
         <v>21</v>
       </c>
@@ -726,11 +741,11 @@
       <c r="D16" s="10">
         <v>12.4</v>
       </c>
-      <c r="E16" s="7" t="s">
+      <c r="E16" s="11" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
         <v>23</v>
       </c>
@@ -743,27 +758,27 @@
       <c r="D17" s="10">
         <v>10.8</v>
       </c>
-      <c r="E17" s="7" t="s">
+      <c r="E17" s="11" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="11" t="s">
+      <c r="A18" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="B18" s="11"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="12">
+      <c r="B18" s="12"/>
+      <c r="C18" s="12"/>
+      <c r="D18" s="13">
         <f>SUM(D16:D17)</f>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="11" t="s">
+      <c r="A20" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="B20" s="11"/>
-      <c r="C20" s="11"/>
-      <c r="D20" s="14">
+      <c r="B20" s="12"/>
+      <c r="C20" s="12"/>
+      <c r="D20" s="15">
         <f>D11/(D11+D18)</f>
       </c>
     </row>

</xml_diff>

<commit_message>
Format odometer as whole number in report export
The .1 in the numFmt showed a perpetual .0 since odometer is stored
in whole km, so drop it to #,##0.
</commit_message>
<xml_diff>
--- a/static/templates/home-charging-template.xlsx
+++ b/static/templates/home-charging-template.xlsx
@@ -98,12 +98,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="5">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="$#,##0.00000"/>
-    <numFmt numFmtId="166" formatCode="#,##0.0"/>
-    <numFmt numFmtId="167" formatCode="$#,##0.00"/>
-    <numFmt numFmtId="168" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="167" formatCode="0.0%"/>
   </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
@@ -197,7 +196,7 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -210,8 +209,8 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="4" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="167" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>

</xml_diff>

<commit_message>
Colorize percentage-of-home row and unify totals styling in report export
Style the "Percentage of Home Charging" summary row and the table total
rows (home kWh, cost, public kWh) to match the teal section banding used
elsewhere in the xlsx export, with consistent row heights. Also fixes the
starting/closing date value cells to stay left-aligned.
</commit_message>
<xml_diff>
--- a/static/templates/home-charging-template.xlsx
+++ b/static/templates/home-charging-template.xlsx
@@ -127,6 +127,8 @@
     </font>
     <font>
       <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="16"/>
     </font>
   </fonts>
   <fills count="4">
@@ -174,10 +176,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -205,12 +209,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="4" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -681,7 +695,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
         <v>18</v>
       </c>
@@ -691,7 +705,7 @@
         <f>SUM(D8:D10)</f>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
         <v>19</v>
       </c>
@@ -761,7 +775,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="12" t="s">
         <v>25</v>
       </c>
@@ -771,15 +785,16 @@
         <f>SUM(D16:D17)</f>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="12" t="s">
+    <row r="20" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="B20" s="12"/>
-      <c r="C20" s="12"/>
-      <c r="D20" s="15">
+      <c r="B20" s="15"/>
+      <c r="C20" s="15"/>
+      <c r="D20" s="16">
         <f>D11/(D11+D18)</f>
       </c>
+      <c r="E20" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>

<commit_message>
Add footer to the sample xlsx template generator for parity
The real footer is written by report.ts at runtime (rows below the header
block get cleared and rebuilt per period), but the checked-in sample
template should still look like a real report if opened directly.
</commit_message>
<xml_diff>
--- a/static/templates/home-charging-template.xlsx
+++ b/static/templates/home-charging-template.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="28">
   <si>
     <t>Full Name:</t>
   </si>
@@ -92,6 +92,9 @@
   </si>
   <si>
     <t>Percentage of Home Charging:</t>
+  </si>
+  <si>
+    <t>Report generated by ev-charging-log — https://github.com/brianramseyau/ev-charging-log</t>
   </si>
 </sst>
 </file>
@@ -104,7 +107,7 @@
     <numFmt numFmtId="166" formatCode="$#,##0.00"/>
     <numFmt numFmtId="167" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -129,6 +132,12 @@
       <b/>
       <color rgb="FFFFFFFF"/>
       <sz val="16"/>
+    </font>
+    <font>
+      <i/>
+      <u/>
+      <color rgb="FF64748B"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="4">
@@ -176,7 +185,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -225,6 +234,9 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -564,7 +576,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -796,15 +808,28 @@
       </c>
       <c r="E20" s="17"/>
     </row>
+    <row r="22" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="B22" s="18"/>
+      <c r="C22" s="18"/>
+      <c r="D22" s="18"/>
+      <c r="E22" s="18"/>
+    </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="A6:E6"/>
     <mergeCell ref="A11:C11"/>
     <mergeCell ref="A12:C12"/>
     <mergeCell ref="A14:E14"/>
     <mergeCell ref="A18:C18"/>
     <mergeCell ref="A20:C20"/>
+    <mergeCell ref="A22:E22"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="A22" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Add footer with repository link to generated reports (#10)
* Add branded footer to xlsx report export

Every generated report now ends with a muted, theme-matching footer row
linking back to the project's GitHub repo.

* Add footer to the sample xlsx template generator for parity

The real footer is written by report.ts at runtime (rows below the header
block get cleared and rebuilt per period), but the checked-in sample
template should still look like a real report if opened directly.

---------

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/static/templates/home-charging-template.xlsx
+++ b/static/templates/home-charging-template.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="28">
   <si>
     <t>Full Name:</t>
   </si>
@@ -92,6 +92,9 @@
   </si>
   <si>
     <t>Percentage of Home Charging:</t>
+  </si>
+  <si>
+    <t>Report generated by ev-charging-log — https://github.com/brianramseyau/ev-charging-log</t>
   </si>
 </sst>
 </file>
@@ -104,7 +107,7 @@
     <numFmt numFmtId="166" formatCode="$#,##0.00"/>
     <numFmt numFmtId="167" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -129,6 +132,12 @@
       <b/>
       <color rgb="FFFFFFFF"/>
       <sz val="16"/>
+    </font>
+    <font>
+      <i/>
+      <u/>
+      <color rgb="FF64748B"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="4">
@@ -176,7 +185,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -225,6 +234,9 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -564,7 +576,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -796,15 +808,28 @@
       </c>
       <c r="E20" s="17"/>
     </row>
+    <row r="22" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="B22" s="18"/>
+      <c r="C22" s="18"/>
+      <c r="D22" s="18"/>
+      <c r="E22" s="18"/>
+    </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="A6:E6"/>
     <mergeCell ref="A11:C11"/>
     <mergeCell ref="A12:C12"/>
     <mergeCell ref="A14:E14"/>
     <mergeCell ref="A18:C18"/>
     <mergeCell ref="A20:C20"/>
+    <mergeCell ref="A22:E22"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="A22" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>